<commit_message>
working on reviewer response 3/19
</commit_message>
<xml_diff>
--- a/Outputs/Annotation/QC.xlsx
+++ b/Outputs/Annotation/QC.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10303"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jdp2019/Desktop/DTC-metabolomics-2026/Outputs/Annotation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/JoshsMacbook2015/Desktop/Repos/DTC-metabolomics-2026/Outputs/Annotation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3078589D-B964-BA46-85D1-25B1CC000219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5393ED0B-6DD8-1141-9B39-CFD0069AC4D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="39120" windowHeight="17820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="QC" sheetId="3" r:id="rId1"/>
@@ -20,7 +20,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Abbreviations!$A$1:$G$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Exclude!$A$1:$U$167</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">QC!$A$1:$Z$132</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">QC!$A$1:$Z$133</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4011" uniqueCount="1625">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4026" uniqueCount="1631">
   <si>
     <t>Identified Name</t>
   </si>
@@ -4915,6 +4915,24 @@
   </si>
   <si>
     <t>Butyrylcarnitine (Butanoylcarnitine)</t>
+  </si>
+  <si>
+    <t>S-Adenosyl-L-methionine</t>
+  </si>
+  <si>
+    <t>HILIC_399.144594130272_111.030810687756</t>
+  </si>
+  <si>
+    <t>C15H22N6O5S</t>
+  </si>
+  <si>
+    <t>C00019</t>
+  </si>
+  <si>
+    <t>HMDB0001185</t>
+  </si>
+  <si>
+    <t>S-Adenosyl-L-methionine (SAM)</t>
   </si>
 </sst>
 </file>
@@ -5351,7 +5369,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{624A435F-8BE2-214B-91C7-3973CD222FA7}">
-  <dimension ref="A1:Z132"/>
+  <dimension ref="A1:Z133"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="38.6640625" bestFit="1" customWidth="1"/>
@@ -14895,13 +14913,81 @@
       </c>
       <c r="Z132" s="3"/>
     </row>
+    <row r="133" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A133" s="3" t="s">
+        <v>1626</v>
+      </c>
+      <c r="B133" s="3" t="s">
+        <v>1590</v>
+      </c>
+      <c r="C133" s="3" t="s">
+        <v>1625</v>
+      </c>
+      <c r="D133" s="3" t="s">
+        <v>1630</v>
+      </c>
+      <c r="E133" s="3" t="s">
+        <v>1590</v>
+      </c>
+      <c r="F133" s="3" t="s">
+        <v>1510</v>
+      </c>
+      <c r="G133" s="3" t="s">
+        <v>1386</v>
+      </c>
+      <c r="H133" s="3">
+        <v>-0.22315655929841999</v>
+      </c>
+      <c r="I133" s="3">
+        <v>0.76393420180305105</v>
+      </c>
+      <c r="J133" s="3"/>
+      <c r="K133" s="3"/>
+      <c r="L133" s="3"/>
+      <c r="M133" s="3"/>
+      <c r="N133" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="O133" s="3">
+        <v>0.915916900898605</v>
+      </c>
+      <c r="P133" s="3">
+        <v>399.14460000000003</v>
+      </c>
+      <c r="Q133" s="3">
+        <v>111</v>
+      </c>
+      <c r="R133" s="3" t="s">
+        <v>603</v>
+      </c>
+      <c r="S133" s="3" t="s">
+        <v>604</v>
+      </c>
+      <c r="T133" s="3" t="s">
+        <v>605</v>
+      </c>
+      <c r="U133" s="3">
+        <v>398.13720000000001</v>
+      </c>
+      <c r="V133" s="3" t="s">
+        <v>1627</v>
+      </c>
+      <c r="W133" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="X133" s="3" t="s">
+        <v>1628</v>
+      </c>
+      <c r="Y133" s="3">
+        <v>34755</v>
+      </c>
+      <c r="Z133" s="3" t="s">
+        <v>1629</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Z132" xr:uid="{624A435F-8BE2-214B-91C7-3973CD222FA7}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Z132">
-      <sortCondition ref="L1:L132"/>
-    </sortState>
-  </autoFilter>
-  <conditionalFormatting sqref="C1:C1048576">
+  <autoFilter ref="A1:Z133" xr:uid="{624A435F-8BE2-214B-91C7-3973CD222FA7}"/>
+  <conditionalFormatting sqref="C137 H133 C1:C132 C140:C1048576 C134">
     <cfRule type="duplicateValues" dxfId="5" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>